<commit_message>
Adding timeslices to wind onshore
</commit_message>
<xml_diff>
--- a/Sets-DemoModels.xlsx
+++ b/Sets-DemoModels.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\DemoModels\DemoS_004\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B36F05B-3127-42C4-8F24-F46AB5B20B3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1003410-CC05-40D0-A57A-BC3515999670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
     <sheet name="VEDA_Sets-Proc" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +24,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -32,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="89">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -293,6 +298,12 @@
   </si>
   <si>
     <t>C_Neg_AndOr</t>
+  </si>
+  <si>
+    <t>ELCWON</t>
+  </si>
+  <si>
+    <t>ELEWON</t>
   </si>
 </sst>
 </file>
@@ -316,7 +327,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -324,12 +335,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1110,7 +1132,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E06336B7-5D6A-48EE-B122-F085391548AD}">
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2853,20 +2875,41 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+    <row r="106" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F106" t="s">
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+      <c r="F106" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H106" t="s">
-        <v>13</v>
-      </c>
-      <c r="I106" t="s">
+      <c r="G106" s="1"/>
+      <c r="H106" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I106" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D107" t="s">
+        <v>87</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H107" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I107" s="2" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding wind offshore's commodity fraction Scenario
</commit_message>
<xml_diff>
--- a/Sets-DemoModels.xlsx
+++ b/Sets-DemoModels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1003410-CC05-40D0-A57A-BC3515999670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9093D5F7-ED35-4FD6-887B-5701C6628D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="91">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -304,6 +304,12 @@
   </si>
   <si>
     <t>ELEWON</t>
+  </si>
+  <si>
+    <t>ELCWOF</t>
+  </si>
+  <si>
+    <t>ELEWOF</t>
   </si>
 </sst>
 </file>
@@ -348,10 +354,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1132,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E06336B7-5D6A-48EE-B122-F085391548AD}">
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2897,19 +2902,36 @@
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A107" s="2" t="s">
+      <c r="A107" t="s">
         <v>14</v>
       </c>
       <c r="D107" t="s">
         <v>87</v>
       </c>
-      <c r="F107" s="2" t="s">
+      <c r="F107" t="s">
         <v>88</v>
       </c>
-      <c r="H107" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I107" s="2" t="s">
+      <c r="H107" t="s">
+        <v>13</v>
+      </c>
+      <c r="I107" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>14</v>
+      </c>
+      <c r="D108" t="s">
+        <v>89</v>
+      </c>
+      <c r="F108" t="s">
+        <v>90</v>
+      </c>
+      <c r="H108" t="s">
+        <v>13</v>
+      </c>
+      <c r="I108" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>